<commit_message>
Add Practice ROI model: planner funnel to firm revenue and client lifetime value
Adds a Practice ROI sheet (3-year revenue, standard vs data-driven approach,
10-year client lifetime value NPV), a chart, and a live Practice ROI tab
in the interactive planner.
</commit_message>
<xml_diff>
--- a/retirement_stress_test_model.xlsx
+++ b/retirement_stress_test_model.xlsx
@@ -15,6 +15,7 @@
     <sheet name="Account Comparison" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Business Cash Flow" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="Simulation" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Practice ROI" sheetId="8" state="visible" r:id="rId10"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -48,7 +49,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="259" uniqueCount="191">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="338" uniqueCount="262">
   <si>
     <t xml:space="preserve">Client Plan Dashboard</t>
   </si>
@@ -86,6 +87,9 @@
     <t xml:space="preserve">Best place for the next dollar</t>
   </si>
   <si>
+    <t xml:space="preserve">Practice: extra 3-year revenue (data-driven)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Retirement Portfolio Stress Test Model</t>
   </si>
   <si>
@@ -621,13 +625,223 @@
   </si>
   <si>
     <t xml:space="preserve">90th pct ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Practice ROI Model: From Planning Conversations to Firm Revenue</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Illustrative assumptions; replace with the firm's figures. Blue = input, green = link, yellow = the four inputs the data-driven approach changes.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Input</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Standard approach</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data-driven approach</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Prospects met per month</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seminars, referrals and meetings</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Conversion to client (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumption: stress test + live planner give prospects a clear reason to act</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annual client retention (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumption: clients who understand their plan stay longer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Average assets per new client ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Increase Consultants averages about $32.9K per client (AdvizorPro)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New contributions per client per year ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ongoing savings added to managed accounts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Portfolio growth before fee (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linked: selected portfolio from the stress-test model</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Linked from Assumptions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clients buying an annuity (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumption: stress test shows when guaranteed income helps</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Average annuity premium ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumption</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annuity commission (% of premium)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumption; varies by product</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clients buying life insurance (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Average annual life premium ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">First-year commission (% of premium)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumption; varies by carrier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Renewal commission (% of premium)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planner cost per year ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assumption: base pay plus licensing and tools</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Discount rate for client value (%)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Used in the lifetime-value DCF</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metric</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Standard Y1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Standard Y2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Standard Y3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data-driven Y1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data-driven Y2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data-driven Y3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">New clients</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clients at year end</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insured clients at year end</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assets under management, year end ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Average AUM during year ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Advisory fee revenue ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Annuity commissions ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insurance first-year commissions ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Insurance renewal commissions ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total revenue ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Planner cost ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Net contribution to firm ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revenue per $1 of planner cost</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3-year summary</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Standard</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data-driven</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Difference</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total revenue, 3 years ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Net contribution, 3 years ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Clients at end of year 3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Assets under management, end of year 3 ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Revenue per $1 of planner cost, 3 years</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data-driven approach changes only conversion, retention, annuity and insurance take-up (yellow cells); everything else is identical, so the difference isolates their effect.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Client lifetime value (one new client)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Standard ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data-driven ($)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Expected cash flow</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lifetime value (NPV of 10 years)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Value of one year's new clients</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Cash flow = survival (retention ^ years) x fee on the client's growing assets, plus expected annuity and first-year insurance commissions in year 1 and insurance renewals after. Excel NPV discounts year-end flows.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="9">
+  <numFmts count="10">
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="0.0%;\(0.0%\);\-"/>
     <numFmt numFmtId="166" formatCode="\$#,##0;&quot;($&quot;#,##0\);\-"/>
@@ -637,6 +851,7 @@
     <numFmt numFmtId="170" formatCode="General"/>
     <numFmt numFmtId="171" formatCode="0"/>
     <numFmt numFmtId="172" formatCode="#,##0"/>
+    <numFmt numFmtId="173" formatCode="0.0\x"/>
   </numFmts>
   <fonts count="16">
     <font>
@@ -797,7 +1012,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="34">
+  <cellXfs count="39">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -934,6 +1149,26 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="172" fontId="12" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="166" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="172" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="173" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1472,11 +1707,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="9559716"/>
-        <c:axId val="11127812"/>
+        <c:axId val="53008298"/>
+        <c:axId val="45516"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="9559716"/>
+        <c:axId val="53008298"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1542,7 +1777,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="11127812"/>
+        <c:crossAx val="45516"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -1550,7 +1785,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="11127812"/>
+        <c:axId val="45516"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -1626,7 +1861,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="9559716"/>
+        <c:crossAx val="53008298"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2003,11 +2238,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="28599085"/>
-        <c:axId val="66032040"/>
+        <c:axId val="8450220"/>
+        <c:axId val="31534961"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="28599085"/>
+        <c:axId val="8450220"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2039,7 +2274,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="66032040"/>
+        <c:crossAx val="31534961"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2047,7 +2282,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="66032040"/>
+        <c:axId val="31534961"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2123,7 +2358,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="28599085"/>
+        <c:crossAx val="8450220"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -2312,11 +2547,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="85896510"/>
-        <c:axId val="81827354"/>
+        <c:axId val="92242416"/>
+        <c:axId val="69356303"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="85896510"/>
+        <c:axId val="92242416"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2348,7 +2583,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="81827354"/>
+        <c:crossAx val="69356303"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -2356,7 +2591,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="81827354"/>
+        <c:axId val="69356303"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -2432,7 +2667,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="85896510"/>
+        <c:crossAx val="92242416"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -3376,11 +3611,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="30296328"/>
-        <c:axId val="61580721"/>
+        <c:axId val="5968466"/>
+        <c:axId val="32959632"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="30296328"/>
+        <c:axId val="5968466"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3446,7 +3681,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61580721"/>
+        <c:crossAx val="32959632"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -3454,7 +3689,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="61580721"/>
+        <c:axId val="32959632"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -3530,7 +3765,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="30296328"/>
+        <c:crossAx val="5968466"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -4714,11 +4949,11 @@
           </c:spPr>
         </c:hiLowLines>
         <c:marker val="0"/>
-        <c:axId val="53982327"/>
-        <c:axId val="61995449"/>
+        <c:axId val="37397644"/>
+        <c:axId val="62203907"/>
       </c:lineChart>
       <c:catAx>
-        <c:axId val="53982327"/>
+        <c:axId val="37397644"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4784,7 +5019,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="61995449"/>
+        <c:crossAx val="62203907"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -4792,7 +5027,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="61995449"/>
+        <c:axId val="62203907"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -4834,7 +5069,372 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="53982327"/>
+        <c:crossAx val="37397644"/>
+        <c:crosses val="autoZero"/>
+        <c:crossBetween val="between"/>
+      </c:valAx>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:plotArea>
+    <c:legend>
+      <c:legendPos val="b"/>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+      <c:txPr>
+        <a:bodyPr/>
+        <a:lstStyle/>
+        <a:p>
+          <a:pPr>
+            <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+              <a:solidFill>
+                <a:srgbClr val="000000"/>
+              </a:solidFill>
+              <a:latin typeface="Calibri"/>
+            </a:defRPr>
+          </a:pPr>
+        </a:p>
+      </c:txPr>
+    </c:legend>
+    <c:plotVisOnly val="1"/>
+    <c:dispBlanksAs val="gap"/>
+  </c:chart>
+  <c:spPr>
+    <a:solidFill>
+      <a:srgbClr val="ffffff"/>
+    </a:solidFill>
+    <a:ln w="9360">
+      <a:solidFill>
+        <a:srgbClr val="d9d9d9"/>
+      </a:solidFill>
+      <a:round/>
+    </a:ln>
+  </c:spPr>
+</c:chartSpace>
+</file>
+
+<file path=xl/charts/chart6.xml><?xml version="1.0" encoding="utf-8"?>
+<c:chartSpace xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <c:lang val="en-US"/>
+  <c:roundedCorners val="0"/>
+  <c:chart>
+    <c:title>
+      <c:tx>
+        <c:rich>
+          <a:bodyPr rot="0"/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+            <a:r>
+              <a:rPr b="1" sz="1800" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:rPr>
+              <a:t>Total revenue by year: standard vs data-driven</a:t>
+            </a:r>
+          </a:p>
+        </c:rich>
+      </c:tx>
+      <c:overlay val="0"/>
+      <c:spPr>
+        <a:noFill/>
+        <a:ln w="0">
+          <a:noFill/>
+        </a:ln>
+      </c:spPr>
+    </c:title>
+    <c:autoTitleDeleted val="0"/>
+    <c:plotArea>
+      <c:barChart>
+        <c:barDir val="col"/>
+        <c:grouping val="clustered"/>
+        <c:varyColors val="0"/>
+        <c:ser>
+          <c:idx val="0"/>
+          <c:order val="0"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"Standard"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Standard</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="4f81bd"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:multiLvlStrRef>
+              <c:f>'Practice ROI'!$B$22:$D$22</c:f>
+              <c:multiLvlStrCache>
+                <c:ptCount val="1"/>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>Standard Y3</c:v>
+                  </c:pt>
+                </c:lvl>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>Standard Y2</c:v>
+                  </c:pt>
+                </c:lvl>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>Standard Y1</c:v>
+                  </c:pt>
+                </c:lvl>
+              </c:multiLvlStrCache>
+            </c:multiLvlStrRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Practice ROI'!$B$32:$D$32</c:f>
+              <c:numCache>
+                <c:formatCode>\$#,##0;"($"#,##0\);\-</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>35820</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>51276.52719</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>68172.4945625706</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
+          <c:tx>
+            <c:strRef>
+              <c:f>"Data-driven"</c:f>
+              <c:strCache>
+                <c:ptCount val="1"/>
+                <c:pt idx="0">
+                  <c:v>Data-driven</c:v>
+                </c:pt>
+              </c:strCache>
+            </c:strRef>
+          </c:tx>
+          <c:spPr>
+            <a:solidFill>
+              <a:srgbClr val="c0504d"/>
+            </a:solidFill>
+            <a:ln w="0">
+              <a:noFill/>
+            </a:ln>
+          </c:spPr>
+          <c:invertIfNegative val="0"/>
+          <c:dLbls>
+            <c:txPr>
+              <a:bodyPr wrap="none"/>
+              <a:lstStyle/>
+              <a:p>
+                <a:pPr>
+                  <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                    <a:latin typeface="Arial"/>
+                  </a:defRPr>
+                </a:pPr>
+              </a:p>
+            </c:txPr>
+            <c:showLegendKey val="0"/>
+            <c:showVal val="0"/>
+            <c:showCatName val="0"/>
+            <c:showSerName val="0"/>
+            <c:showPercent val="0"/>
+            <c:separator> </c:separator>
+            <c:showLeaderLines val="1"/>
+            <c:extLst>
+              <c:ext xmlns:c15="http://schemas.microsoft.com/office/drawing/2012/chart" uri="{CE6537A1-D6FC-4f65-9D91-7224C49458BB}">
+                <c15:showLeaderLines val="1"/>
+              </c:ext>
+            </c:extLst>
+          </c:dLbls>
+          <c:cat>
+            <c:multiLvlStrRef>
+              <c:f>'Practice ROI'!$B$22:$D$22</c:f>
+              <c:multiLvlStrCache>
+                <c:ptCount val="1"/>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>Standard Y3</c:v>
+                  </c:pt>
+                </c:lvl>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>Standard Y2</c:v>
+                  </c:pt>
+                </c:lvl>
+                <c:lvl>
+                  <c:pt idx="0">
+                    <c:v>Standard Y1</c:v>
+                  </c:pt>
+                </c:lvl>
+              </c:multiLvlStrCache>
+            </c:multiLvlStrRef>
+          </c:cat>
+          <c:val>
+            <c:numRef>
+              <c:f>'Practice ROI'!$E$32:$G$32</c:f>
+              <c:numCache>
+                <c:formatCode>\$#,##0;"($"#,##0\);\-</c:formatCode>
+                <c:ptCount val="3"/>
+                <c:pt idx="0">
+                  <c:v>56640</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>77786.50845</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>101619.19794091</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:val>
+        </c:ser>
+        <c:gapWidth val="150"/>
+        <c:overlap val="0"/>
+        <c:axId val="18989738"/>
+        <c:axId val="46914933"/>
+      </c:barChart>
+      <c:catAx>
+        <c:axId val="18989738"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="b"/>
+        <c:numFmt formatCode="General" sourceLinked="1"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="46914933"/>
+        <c:crosses val="autoZero"/>
+        <c:auto val="1"/>
+        <c:lblAlgn val="ctr"/>
+        <c:lblOffset val="100"/>
+        <c:noMultiLvlLbl val="0"/>
+      </c:catAx>
+      <c:valAx>
+        <c:axId val="46914933"/>
+        <c:scaling>
+          <c:orientation val="minMax"/>
+        </c:scaling>
+        <c:delete val="0"/>
+        <c:axPos val="l"/>
+        <c:majorGridlines>
+          <c:spPr>
+            <a:ln w="9360">
+              <a:solidFill>
+                <a:srgbClr val="878787"/>
+              </a:solidFill>
+              <a:round/>
+            </a:ln>
+          </c:spPr>
+        </c:majorGridlines>
+        <c:numFmt formatCode="\$#,##0" sourceLinked="0"/>
+        <c:majorTickMark val="none"/>
+        <c:minorTickMark val="none"/>
+        <c:tickLblPos val="nextTo"/>
+        <c:spPr>
+          <a:ln w="9360">
+            <a:solidFill>
+              <a:srgbClr val="878787"/>
+            </a:solidFill>
+            <a:round/>
+          </a:ln>
+        </c:spPr>
+        <c:txPr>
+          <a:bodyPr/>
+          <a:lstStyle/>
+          <a:p>
+            <a:pPr>
+              <a:defRPr b="0" sz="1000" spc="-1" strike="noStrike">
+                <a:solidFill>
+                  <a:srgbClr val="000000"/>
+                </a:solidFill>
+                <a:latin typeface="Calibri"/>
+              </a:defRPr>
+            </a:pPr>
+          </a:p>
+        </c:txPr>
+        <c:crossAx val="18989738"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>
@@ -5056,6 +5656,41 @@
 </xdr:wsDr>
 </file>
 
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>2</xdr:row>
+      <xdr:rowOff>160920</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>17</xdr:col>
+      <xdr:colOff>256320</xdr:colOff>
+      <xdr:row>17</xdr:row>
+      <xdr:rowOff>32400</xdr:rowOff>
+    </xdr:to>
+    <xdr:graphicFrame>
+      <xdr:nvGraphicFramePr>
+        <xdr:cNvPr id="5" name="Chart 1"/>
+        <xdr:cNvGraphicFramePr/>
+      </xdr:nvGraphicFramePr>
+      <xdr:xfrm>
+        <a:off x="11113920" y="571680"/>
+        <a:ext cx="5759640" cy="2879640"/>
+      </xdr:xfrm>
+      <a:graphic>
+        <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+        </a:graphicData>
+      </a:graphic>
+    </xdr:graphicFrame>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+</xdr:wsDr>
+</file>
+
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
 <a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Office Theme">
   <a:themeElements>
@@ -5236,7 +5871,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="36"/>
@@ -5331,6 +5966,15 @@
       <c r="B13" s="5" t="str">
         <f aca="false">'Account Comparison'!B31</f>
         <v>401(k) with employer match</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="B14" s="7" t="n">
+        <f aca="false">'Practice ROI'!D38</f>
+        <v>80776.6846383398</v>
       </c>
     </row>
   </sheetData>
@@ -5361,39 +6005,39 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="3" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B3" s="3" t="s">
         <v>3</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B4" s="8" t="n">
         <v>35</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B5" s="8" t="n">
         <v>65</v>
@@ -5402,18 +6046,18 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="B6" s="8" t="n">
         <v>92</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B7" s="9" t="n">
         <v>50000</v>
@@ -5422,40 +6066,40 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B8" s="9" t="n">
         <v>12000</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B9" s="10" t="n">
         <v>0.03</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B10" s="10" t="n">
         <v>0.025</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B11" s="9" t="n">
         <v>50000</v>
@@ -5464,62 +6108,62 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B12" s="9" t="n">
         <v>24000</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="4" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B13" s="10" t="n">
         <v>0.01</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="3" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B15" s="3" t="s">
         <v>3</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B16" s="11" t="n">
         <v>2</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B17" s="12" t="n">
         <v>0.05</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="B18" s="0" t="str">
         <f aca="false">INDEX($E$21:$G$21,1,$B$16)</f>
@@ -5528,47 +6172,47 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="3" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="F20" s="3" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="G20" s="3" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="13" t="s">
+        <v>47</v>
+      </c>
+      <c r="E21" s="13" t="s">
+        <v>44</v>
+      </c>
+      <c r="F21" s="13" t="s">
+        <v>45</v>
+      </c>
+      <c r="G21" s="13" t="s">
         <v>46</v>
-      </c>
-      <c r="E21" s="13" t="s">
-        <v>43</v>
-      </c>
-      <c r="F21" s="13" t="s">
-        <v>44</v>
-      </c>
-      <c r="G21" s="13" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B22" s="4" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C22" s="10" t="n">
         <v>0.07</v>
@@ -5588,10 +6232,10 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="C23" s="10" t="n">
         <v>0.065</v>
@@ -5611,10 +6255,10 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="4" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B24" s="4" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="C24" s="10" t="n">
         <v>0.04</v>
@@ -5634,10 +6278,10 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="4" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="B25" s="4" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="C25" s="10" t="n">
         <v>0.038</v>
@@ -5657,7 +6301,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E26" s="14" t="n">
         <f aca="false">SUM(E22:E25)</f>
@@ -5674,24 +6318,24 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B28" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B29" s="15" t="n">
         <v>1</v>
@@ -5708,7 +6352,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="13" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B30" s="15" t="n">
         <v>0.8</v>
@@ -5725,7 +6369,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B31" s="15" t="n">
         <v>0.1</v>
@@ -5742,7 +6386,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B32" s="15" t="n">
         <v>0.1</v>
@@ -5759,24 +6403,24 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
+        <v>60</v>
+      </c>
+      <c r="B34" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>58</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>52</v>
+      </c>
+      <c r="E34" s="3" t="s">
         <v>59</v>
-      </c>
-      <c r="B34" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="C34" s="3" t="s">
-        <v>57</v>
-      </c>
-      <c r="D34" s="3" t="s">
-        <v>51</v>
-      </c>
-      <c r="E34" s="3" t="s">
-        <v>58</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="13" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="B35" s="16" t="n">
         <f aca="false">$D$22*$D$22*B29</f>
@@ -5797,7 +6441,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="13" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="B36" s="16" t="n">
         <f aca="false">$D$23*$D$22*B30</f>
@@ -5818,7 +6462,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="B37" s="16" t="n">
         <f aca="false">$D$24*$D$22*B31</f>
@@ -5839,7 +6483,7 @@
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A38" s="13" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="B38" s="16" t="n">
         <f aca="false">$D$25*$D$22*B32</f>
@@ -5860,7 +6504,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
     </row>
   </sheetData>
@@ -5891,41 +6535,41 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="52.2" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B4" s="3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="I4" s="3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="J4" s="3" t="s">
         <v>8</v>
@@ -5934,16 +6578,16 @@
         <v>9</v>
       </c>
       <c r="L4" s="3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="M4" s="3" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="N4" s="3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="Q4" s="13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -6003,7 +6647,7 @@
         <v>-1098509.47838456</v>
       </c>
       <c r="Q5" s="4" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="R5" s="17" t="n">
         <f aca="false">Assumptions!B5-Assumptions!B4</f>
@@ -6067,7 +6711,7 @@
         <v>-1100758.60370974</v>
       </c>
       <c r="Q6" s="4" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="R6" s="17" t="n">
         <f aca="false">Assumptions!B6-Assumptions!B5</f>
@@ -6131,7 +6775,7 @@
         <v>-1103726.80365842</v>
       </c>
       <c r="Q7" s="4" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="R7" s="21" t="n">
         <f aca="false">(Assumptions!B11-Assumptions!B12)*(1+Assumptions!B10)^R5</f>
@@ -6482,14 +7126,14 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="B15" s="22" t="n">
         <f aca="false">(Assumptions!B16-1)*3+MATCH(Assumptions!B17,B5:B7,0)</f>
         <v>5</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
     </row>
   </sheetData>
@@ -6520,26 +7164,26 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="0" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B2" s="17" t="str">
         <f aca="false">Assumptions!B18</f>
         <v>Balanced</v>
       </c>
       <c r="D2" s="22" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E2" s="23" t="n">
         <f aca="false">Assumptions!B17</f>
         <v>0.05</v>
       </c>
       <c r="G2" s="22" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="H2" s="19" t="n">
         <f aca="false">SUMPRODUCT(INDEX(Assumptions!$E$22:$G$24,0,Assumptions!$B$16),Assumptions!$C$22:$C$24)*(1-Assumptions!$B$17)+Assumptions!$B$17*Assumptions!$C$25-Assumptions!$B$13</f>
@@ -6548,7 +7192,7 @@
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="G3" s="0" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="H3" s="21" t="n">
         <f aca="false">Scenarios!R7</f>
@@ -6557,28 +7201,28 @@
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="3" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B5" s="3" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E5" s="3" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -8544,186 +9188,186 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="B5" s="9" t="n">
         <v>7500</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B6" s="10" t="n">
         <v>0.22</v>
       </c>
       <c r="C6" s="2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="B7" s="12" t="n">
         <v>0.12</v>
       </c>
       <c r="C7" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="B8" s="10" t="n">
         <v>0.15</v>
       </c>
       <c r="C8" s="2" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="B9" s="10" t="n">
         <v>0.005</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="B10" s="9" t="n">
         <v>75000</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B11" s="10" t="n">
         <v>0.5</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="B12" s="10" t="n">
         <v>0.06</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B14" s="3" t="s">
         <v>3</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="B15" s="24" t="n">
         <f aca="false">Assumptions!B5-Assumptions!B4</f>
         <v>30</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="B16" s="23" t="n">
         <f aca="false">Projection!H2</f>
         <v>0.0462875</v>
       </c>
       <c r="C16" s="2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="B17" s="23" t="n">
         <f aca="false">Assumptions!B9</f>
         <v>0.03</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="3" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B19" s="3" t="s">
         <v>3</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="4" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B20" s="25" t="n">
         <f aca="false">IF(ABS(B16-B17)&lt;0.000001,B15*(1+B16)^(B15-1),((1+B16)^B15-(1+B17)^B15)/(B16-B17))</f>
         <v>89.5773347126353</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="4" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B21" s="25" t="n">
         <f aca="false">IF(ABS((B16-B9)-B17)&lt;0.000001,B15*(1+B16-B9)^(B15-1),((1+B16-B9)^B15-(1+B17)^B15)/((B16-B9)-B17))</f>
@@ -8732,7 +9376,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="4" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="B22" s="25" t="n">
         <f aca="false">IF(B17=0,B15,((1+B17)^B15-1)/B17)</f>
@@ -8741,7 +9385,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="4" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="B23" s="20" t="n">
         <f aca="false">B11*MIN(B5,B12*B10)</f>
@@ -8750,33 +9394,33 @@
     </row>
     <row r="25" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="3" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B25" s="3" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>8</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="G25" s="3" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="13" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B26" s="26" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C26" s="20" t="n">
         <f aca="false">B5*(1-B6)</f>
@@ -8801,10 +9445,10 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="13" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="B27" s="26" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="C27" s="20" t="n">
         <f aca="false">B5</f>
@@ -8829,10 +9473,10 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="13" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="B28" s="26" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="C28" s="20" t="n">
         <f aca="false">B5*(1-B6)</f>
@@ -8857,10 +9501,10 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="13" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B29" s="26" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="C29" s="20" t="n">
         <f aca="false">B5+B23</f>
@@ -8885,7 +9529,7 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="13" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B31" s="0" t="str">
         <f aca="false">INDEX(A26:A29,MATCH(MAX(F26:F29),F26:F29,0))</f>
@@ -8894,7 +9538,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="13" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B32" s="0" t="str">
         <f aca="false">IF(F27&gt;F28,"Traditional IRA",IF(F28&gt;F27,"Roth IRA","Tie"))</f>
@@ -8903,19 +9547,19 @@
     </row>
     <row r="34" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="3" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="B34" s="3" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -9025,7 +9669,7 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
     </row>
   </sheetData>
@@ -9056,46 +9700,46 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>3</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="E4" s="3" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="G4" s="3" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="B5" s="9" t="n">
         <v>300000</v>
       </c>
       <c r="D5" s="13" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="E5" s="10" t="n">
         <v>0</v>
@@ -9114,13 +9758,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B6" s="27" t="n">
         <v>250</v>
       </c>
       <c r="D6" s="13" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="E6" s="10" t="n">
         <v>0.1</v>
@@ -9139,13 +9783,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="B7" s="9" t="n">
         <v>150</v>
       </c>
       <c r="D7" s="13" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E7" s="10" t="n">
         <v>0</v>
@@ -9164,13 +9808,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="B8" s="10" t="n">
         <v>0.05</v>
       </c>
       <c r="D8" s="13" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E8" s="10" t="n">
         <v>0</v>
@@ -9187,7 +9831,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B9" s="10" t="n">
         <v>0.02</v>
@@ -9195,18 +9839,18 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B10" s="10" t="n">
         <v>0.25</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="4" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B11" s="9" t="n">
         <v>45000</v>
@@ -9214,27 +9858,27 @@
     </row>
     <row r="12" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="3" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="E12" s="3" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F12" s="3" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="13" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B13" s="28" t="n">
         <f aca="false">C44</f>
@@ -9259,7 +9903,7 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="13" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="B14" s="28" t="n">
         <f aca="false">J44</f>
@@ -9284,7 +9928,7 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="13" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B15" s="28" t="n">
         <f aca="false">Q44</f>
@@ -9309,7 +9953,7 @@
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="13" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B16" s="28" t="n">
         <f aca="false">X44</f>
@@ -9334,113 +9978,113 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="2" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="13" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="B19" s="13" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="I19" s="13" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="P19" s="13" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="W19" s="13" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="30" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="C20" s="3" t="s">
+        <v>172</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>173</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>174</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>175</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>176</v>
+      </c>
+      <c r="H20" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="I20" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="D20" s="3" t="s">
+      <c r="J20" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="E20" s="3" t="s">
+      <c r="K20" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="F20" s="3" t="s">
+      <c r="L20" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="G20" s="3" t="s">
+      <c r="M20" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="H20" s="3" t="s">
+      <c r="N20" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="I20" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="J20" s="3" t="s">
+      <c r="O20" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="P20" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="K20" s="3" t="s">
+      <c r="Q20" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="L20" s="3" t="s">
+      <c r="R20" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="M20" s="3" t="s">
+      <c r="S20" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="N20" s="3" t="s">
+      <c r="T20" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="O20" s="3" t="s">
+      <c r="U20" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="P20" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="Q20" s="3" t="s">
+      <c r="V20" s="3" t="s">
+        <v>177</v>
+      </c>
+      <c r="W20" s="3" t="s">
         <v>171</v>
       </c>
-      <c r="R20" s="3" t="s">
+      <c r="X20" s="3" t="s">
         <v>172</v>
       </c>
-      <c r="S20" s="3" t="s">
+      <c r="Y20" s="3" t="s">
         <v>173</v>
       </c>
-      <c r="T20" s="3" t="s">
+      <c r="Z20" s="3" t="s">
         <v>174</v>
       </c>
-      <c r="U20" s="3" t="s">
+      <c r="AA20" s="3" t="s">
         <v>175</v>
       </c>
-      <c r="V20" s="3" t="s">
+      <c r="AB20" s="3" t="s">
         <v>176</v>
       </c>
-      <c r="W20" s="3" t="s">
-        <v>170</v>
-      </c>
-      <c r="X20" s="3" t="s">
-        <v>171</v>
-      </c>
-      <c r="Y20" s="3" t="s">
-        <v>172</v>
-      </c>
-      <c r="Z20" s="3" t="s">
-        <v>173</v>
-      </c>
-      <c r="AA20" s="3" t="s">
-        <v>174</v>
-      </c>
-      <c r="AB20" s="3" t="s">
-        <v>175</v>
-      </c>
       <c r="AC20" s="3" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12277,17 +12921,17 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="3" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B4" s="3" t="s">
         <v>3</v>
@@ -12295,7 +12939,7 @@
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="4" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B5" s="31" t="n">
         <v>1000</v>
@@ -12303,7 +12947,7 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="4" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B6" s="33" t="n">
         <v>0.88</v>
@@ -12311,7 +12955,7 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="4" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B7" s="18" t="n">
         <v>0.746</v>
@@ -12319,7 +12963,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="4" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B8" s="20" t="n">
         <v>-13994.2561517062</v>
@@ -12327,7 +12971,7 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="4" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="B9" s="20" t="n">
         <v>221752.534258649</v>
@@ -12335,7 +12979,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="4" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="B10" s="20" t="n">
         <v>537479.029202344</v>
@@ -12343,22 +12987,22 @@
     </row>
     <row r="13" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="3" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="E13" s="3" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F13" s="3" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -12839,6 +13483,982 @@
       </c>
       <c r="F37" s="20" t="n">
         <v>537479.029202344</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G59"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="44"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="2" style="0" width="17"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="5" style="0" width="17"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>192</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="3" t="s">
+        <v>194</v>
+      </c>
+      <c r="B4" s="3" t="s">
+        <v>195</v>
+      </c>
+      <c r="C4" s="3" t="s">
+        <v>196</v>
+      </c>
+      <c r="D4" s="3" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="4" t="s">
+        <v>197</v>
+      </c>
+      <c r="B5" s="34" t="n">
+        <v>20</v>
+      </c>
+      <c r="C5" s="34" t="n">
+        <v>20</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="4" t="s">
+        <v>199</v>
+      </c>
+      <c r="B6" s="10" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C6" s="12" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>200</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="B7" s="10" t="n">
+        <v>0.92</v>
+      </c>
+      <c r="C7" s="12" t="n">
+        <v>0.95</v>
+      </c>
+      <c r="D7" s="2" t="s">
+        <v>202</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B8" s="9" t="n">
+        <v>33000</v>
+      </c>
+      <c r="C8" s="9" t="n">
+        <v>33000</v>
+      </c>
+      <c r="D8" s="2" t="s">
+        <v>204</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="B9" s="9" t="n">
+        <v>6000</v>
+      </c>
+      <c r="C9" s="9" t="n">
+        <v>6000</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>206</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="4" t="s">
+        <v>207</v>
+      </c>
+      <c r="B10" s="23" t="n">
+        <f aca="false">Projection!$H$2+Assumptions!$B$13</f>
+        <v>0.0562875</v>
+      </c>
+      <c r="C10" s="23" t="n">
+        <f aca="false">Projection!$H$2+Assumptions!$B$13</f>
+        <v>0.0562875</v>
+      </c>
+      <c r="D10" s="2" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="4" t="s">
+        <v>32</v>
+      </c>
+      <c r="B11" s="23" t="n">
+        <f aca="false">Assumptions!$B$13</f>
+        <v>0.01</v>
+      </c>
+      <c r="C11" s="23" t="n">
+        <f aca="false">Assumptions!$B$13</f>
+        <v>0.01</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="4" t="s">
+        <v>210</v>
+      </c>
+      <c r="B12" s="10" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C12" s="12" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>50000</v>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>50000</v>
+      </c>
+      <c r="D13" s="2" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="B14" s="10" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C14" s="10" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D14" s="2" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="B15" s="10" t="n">
+        <v>0.25</v>
+      </c>
+      <c r="C15" s="12" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="D15" s="2" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="B16" s="9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="C16" s="9" t="n">
+        <v>1500</v>
+      </c>
+      <c r="D16" s="2" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="B17" s="10" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="C17" s="10" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="D17" s="2" t="s">
+        <v>219</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="4" t="s">
+        <v>220</v>
+      </c>
+      <c r="B18" s="10" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C18" s="10" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="D18" s="2" t="s">
+        <v>213</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="B19" s="9" t="n">
+        <v>45000</v>
+      </c>
+      <c r="C19" s="9" t="n">
+        <v>45000</v>
+      </c>
+      <c r="D19" s="2" t="s">
+        <v>222</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="4" t="s">
+        <v>223</v>
+      </c>
+      <c r="B20" s="10" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="C20" s="10" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="3" t="s">
+        <v>225</v>
+      </c>
+      <c r="B22" s="3" t="s">
+        <v>226</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>227</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>228</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>229</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>230</v>
+      </c>
+      <c r="G22" s="3" t="s">
+        <v>231</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="4" t="s">
+        <v>232</v>
+      </c>
+      <c r="B23" s="31" t="n">
+        <f aca="false">$B$5*12*$B$6</f>
+        <v>36</v>
+      </c>
+      <c r="C23" s="31" t="n">
+        <f aca="false">$B$5*12*$B$6</f>
+        <v>36</v>
+      </c>
+      <c r="D23" s="31" t="n">
+        <f aca="false">$B$5*12*$B$6</f>
+        <v>36</v>
+      </c>
+      <c r="E23" s="31" t="n">
+        <f aca="false">$C$5*12*$C$6</f>
+        <v>48</v>
+      </c>
+      <c r="F23" s="31" t="n">
+        <f aca="false">$C$5*12*$C$6</f>
+        <v>48</v>
+      </c>
+      <c r="G23" s="31" t="n">
+        <f aca="false">$C$5*12*$C$6</f>
+        <v>48</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="B24" s="31" t="n">
+        <f aca="false">0*$B$7+B23</f>
+        <v>36</v>
+      </c>
+      <c r="C24" s="31" t="n">
+        <f aca="false">B24*$B$7+C23</f>
+        <v>69.12</v>
+      </c>
+      <c r="D24" s="31" t="n">
+        <f aca="false">C24*$B$7+D23</f>
+        <v>99.5904</v>
+      </c>
+      <c r="E24" s="31" t="n">
+        <f aca="false">0*$C$7+E23</f>
+        <v>48</v>
+      </c>
+      <c r="F24" s="31" t="n">
+        <f aca="false">E24*$C$7+F23</f>
+        <v>93.6</v>
+      </c>
+      <c r="G24" s="31" t="n">
+        <f aca="false">F24*$C$7+G23</f>
+        <v>136.92</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="4" t="s">
+        <v>234</v>
+      </c>
+      <c r="B25" s="31" t="n">
+        <f aca="false">0*$B$7+B23*$B$15</f>
+        <v>9</v>
+      </c>
+      <c r="C25" s="31" t="n">
+        <f aca="false">B25*$B$7+C23*$B$15</f>
+        <v>17.28</v>
+      </c>
+      <c r="D25" s="31" t="n">
+        <f aca="false">C25*$B$7+D23*$B$15</f>
+        <v>24.8976</v>
+      </c>
+      <c r="E25" s="31" t="n">
+        <f aca="false">0*$C$7+E23*$C$15</f>
+        <v>14.4</v>
+      </c>
+      <c r="F25" s="31" t="n">
+        <f aca="false">E25*$C$7+F23*$C$15</f>
+        <v>28.08</v>
+      </c>
+      <c r="G25" s="31" t="n">
+        <f aca="false">F25*$C$7+G23*$C$15</f>
+        <v>41.076</v>
+      </c>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="B26" s="20" t="n">
+        <f aca="false">0*$B$7*(1+$B$10)+B23*$B$8+B24*$B$9</f>
+        <v>1404000</v>
+      </c>
+      <c r="C26" s="20" t="n">
+        <f aca="false">B26*$B$7*(1+$B$10)+C23*$B$8+C24*$B$9</f>
+        <v>2967105.438</v>
+      </c>
+      <c r="D26" s="20" t="n">
+        <f aca="false">C26*$B$7*(1+$B$10)+D23*$B$8+D24*$B$9</f>
+        <v>4668929.47451411</v>
+      </c>
+      <c r="E26" s="20" t="n">
+        <f aca="false">0*$C$7*(1+$C$10)+E23*$C$8+E24*$C$9</f>
+        <v>1872000</v>
+      </c>
+      <c r="F26" s="20" t="n">
+        <f aca="false">E26*$C$7*(1+$C$10)+F23*$C$8+F24*$C$9</f>
+        <v>4024101.69</v>
+      </c>
+      <c r="G26" s="20" t="n">
+        <f aca="false">F26*$C$7*(1+$C$10)+G23*$C$8+G24*$C$9</f>
+        <v>6443597.89818208</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="4" t="s">
+        <v>236</v>
+      </c>
+      <c r="B27" s="20" t="n">
+        <f aca="false">(0+B26)/2</f>
+        <v>702000</v>
+      </c>
+      <c r="C27" s="20" t="n">
+        <f aca="false">(B26+C26)/2</f>
+        <v>2185552.719</v>
+      </c>
+      <c r="D27" s="20" t="n">
+        <f aca="false">(C26+D26)/2</f>
+        <v>3818017.45625706</v>
+      </c>
+      <c r="E27" s="20" t="n">
+        <f aca="false">(0+E26)/2</f>
+        <v>936000</v>
+      </c>
+      <c r="F27" s="20" t="n">
+        <f aca="false">(E26+F26)/2</f>
+        <v>2948050.845</v>
+      </c>
+      <c r="G27" s="20" t="n">
+        <f aca="false">(F26+G26)/2</f>
+        <v>5233849.79409104</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="4" t="s">
+        <v>237</v>
+      </c>
+      <c r="B28" s="20" t="n">
+        <f aca="false">B27*$B$11</f>
+        <v>7020</v>
+      </c>
+      <c r="C28" s="20" t="n">
+        <f aca="false">C27*$B$11</f>
+        <v>21855.52719</v>
+      </c>
+      <c r="D28" s="20" t="n">
+        <f aca="false">D27*$B$11</f>
+        <v>38180.1745625706</v>
+      </c>
+      <c r="E28" s="20" t="n">
+        <f aca="false">E27*$C$11</f>
+        <v>9360</v>
+      </c>
+      <c r="F28" s="20" t="n">
+        <f aca="false">F27*$C$11</f>
+        <v>29480.50845</v>
+      </c>
+      <c r="G28" s="20" t="n">
+        <f aca="false">G27*$C$11</f>
+        <v>52338.4979409104</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="4" t="s">
+        <v>238</v>
+      </c>
+      <c r="B29" s="20" t="n">
+        <f aca="false">B23*$B$12*$B$13*$B$14</f>
+        <v>18000</v>
+      </c>
+      <c r="C29" s="20" t="n">
+        <f aca="false">C23*$B$12*$B$13*$B$14</f>
+        <v>18000</v>
+      </c>
+      <c r="D29" s="20" t="n">
+        <f aca="false">D23*$B$12*$B$13*$B$14</f>
+        <v>18000</v>
+      </c>
+      <c r="E29" s="20" t="n">
+        <f aca="false">E23*$C$12*$C$13*$C$14</f>
+        <v>30000</v>
+      </c>
+      <c r="F29" s="20" t="n">
+        <f aca="false">F23*$C$12*$C$13*$C$14</f>
+        <v>30000</v>
+      </c>
+      <c r="G29" s="20" t="n">
+        <f aca="false">G23*$C$12*$C$13*$C$14</f>
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B30" s="20" t="n">
+        <f aca="false">B23*$B$15*$B$16*$B$17</f>
+        <v>10800</v>
+      </c>
+      <c r="C30" s="20" t="n">
+        <f aca="false">C23*$B$15*$B$16*$B$17</f>
+        <v>10800</v>
+      </c>
+      <c r="D30" s="20" t="n">
+        <f aca="false">D23*$B$15*$B$16*$B$17</f>
+        <v>10800</v>
+      </c>
+      <c r="E30" s="20" t="n">
+        <f aca="false">E23*$C$15*$C$16*$C$17</f>
+        <v>17280</v>
+      </c>
+      <c r="F30" s="20" t="n">
+        <f aca="false">F23*$C$15*$C$16*$C$17</f>
+        <v>17280</v>
+      </c>
+      <c r="G30" s="20" t="n">
+        <f aca="false">G23*$C$15*$C$16*$C$17</f>
+        <v>17280</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="B31" s="20" t="n">
+        <f aca="false">0*$B$7*$B$16*$B$18</f>
+        <v>0</v>
+      </c>
+      <c r="C31" s="20" t="n">
+        <f aca="false">B25*$B$7*$B$16*$B$18</f>
+        <v>621</v>
+      </c>
+      <c r="D31" s="20" t="n">
+        <f aca="false">C25*$B$7*$B$16*$B$18</f>
+        <v>1192.32</v>
+      </c>
+      <c r="E31" s="20" t="n">
+        <f aca="false">0*$C$7*$C$16*$C$18</f>
+        <v>0</v>
+      </c>
+      <c r="F31" s="20" t="n">
+        <f aca="false">E25*$C$7*$C$16*$C$18</f>
+        <v>1026</v>
+      </c>
+      <c r="G31" s="20" t="n">
+        <f aca="false">F25*$C$7*$C$16*$C$18</f>
+        <v>2000.7</v>
+      </c>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="13" t="s">
+        <v>241</v>
+      </c>
+      <c r="B32" s="20" t="n">
+        <f aca="false">SUM(B28:B31)</f>
+        <v>35820</v>
+      </c>
+      <c r="C32" s="20" t="n">
+        <f aca="false">SUM(C28:C31)</f>
+        <v>51276.52719</v>
+      </c>
+      <c r="D32" s="20" t="n">
+        <f aca="false">SUM(D28:D31)</f>
+        <v>68172.4945625706</v>
+      </c>
+      <c r="E32" s="20" t="n">
+        <f aca="false">SUM(E28:E31)</f>
+        <v>56640</v>
+      </c>
+      <c r="F32" s="20" t="n">
+        <f aca="false">SUM(F28:F31)</f>
+        <v>77786.50845</v>
+      </c>
+      <c r="G32" s="20" t="n">
+        <f aca="false">SUM(G28:G31)</f>
+        <v>101619.19794091</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="B33" s="20" t="n">
+        <f aca="false">$B$19</f>
+        <v>45000</v>
+      </c>
+      <c r="C33" s="20" t="n">
+        <f aca="false">$B$19</f>
+        <v>45000</v>
+      </c>
+      <c r="D33" s="20" t="n">
+        <f aca="false">$B$19</f>
+        <v>45000</v>
+      </c>
+      <c r="E33" s="20" t="n">
+        <f aca="false">$C$19</f>
+        <v>45000</v>
+      </c>
+      <c r="F33" s="20" t="n">
+        <f aca="false">$C$19</f>
+        <v>45000</v>
+      </c>
+      <c r="G33" s="20" t="n">
+        <f aca="false">$C$19</f>
+        <v>45000</v>
+      </c>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="13" t="s">
+        <v>243</v>
+      </c>
+      <c r="B34" s="20" t="n">
+        <f aca="false">B32-B33</f>
+        <v>-9180</v>
+      </c>
+      <c r="C34" s="20" t="n">
+        <f aca="false">C32-C33</f>
+        <v>6276.52719</v>
+      </c>
+      <c r="D34" s="20" t="n">
+        <f aca="false">D32-D33</f>
+        <v>23172.4945625706</v>
+      </c>
+      <c r="E34" s="20" t="n">
+        <f aca="false">E32-E33</f>
+        <v>11640</v>
+      </c>
+      <c r="F34" s="20" t="n">
+        <f aca="false">F32-F33</f>
+        <v>32786.50845</v>
+      </c>
+      <c r="G34" s="20" t="n">
+        <f aca="false">G32-G33</f>
+        <v>56619.1979409104</v>
+      </c>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="B35" s="35" t="n">
+        <f aca="false">IF(B33=0,0,B32/B33)</f>
+        <v>0.796</v>
+      </c>
+      <c r="C35" s="35" t="n">
+        <f aca="false">IF(C33=0,0,C32/C33)</f>
+        <v>1.139478382</v>
+      </c>
+      <c r="D35" s="35" t="n">
+        <f aca="false">IF(D33=0,0,D32/D33)</f>
+        <v>1.51494432361268</v>
+      </c>
+      <c r="E35" s="35" t="n">
+        <f aca="false">IF(E33=0,0,E32/E33)</f>
+        <v>1.25866666666667</v>
+      </c>
+      <c r="F35" s="35" t="n">
+        <f aca="false">IF(F33=0,0,F32/F33)</f>
+        <v>1.72858907666667</v>
+      </c>
+      <c r="G35" s="35" t="n">
+        <f aca="false">IF(G33=0,0,G32/G33)</f>
+        <v>2.2582043986869</v>
+      </c>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="3" t="s">
+        <v>245</v>
+      </c>
+      <c r="B37" s="3" t="s">
+        <v>246</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>247</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="13" t="s">
+        <v>249</v>
+      </c>
+      <c r="B38" s="20" t="n">
+        <f aca="false">SUM(B32:D32)</f>
+        <v>155269.021752571</v>
+      </c>
+      <c r="C38" s="20" t="n">
+        <f aca="false">SUM(E32:G32)</f>
+        <v>236045.70639091</v>
+      </c>
+      <c r="D38" s="36" t="n">
+        <f aca="false">C38-B38</f>
+        <v>80776.6846383398</v>
+      </c>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="13" t="s">
+        <v>250</v>
+      </c>
+      <c r="B39" s="20" t="n">
+        <f aca="false">SUM(B34:D34)</f>
+        <v>20269.0217525706</v>
+      </c>
+      <c r="C39" s="20" t="n">
+        <f aca="false">SUM(E34:G34)</f>
+        <v>101045.70639091</v>
+      </c>
+      <c r="D39" s="36" t="n">
+        <f aca="false">C39-B39</f>
+        <v>80776.6846383398</v>
+      </c>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="13" t="s">
+        <v>251</v>
+      </c>
+      <c r="B40" s="31" t="n">
+        <f aca="false">D24</f>
+        <v>99.5904</v>
+      </c>
+      <c r="C40" s="31" t="n">
+        <f aca="false">G24</f>
+        <v>136.92</v>
+      </c>
+      <c r="D40" s="37" t="n">
+        <f aca="false">C40-B40</f>
+        <v>37.3296</v>
+      </c>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="13" t="s">
+        <v>252</v>
+      </c>
+      <c r="B41" s="20" t="n">
+        <f aca="false">D26</f>
+        <v>4668929.47451411</v>
+      </c>
+      <c r="C41" s="20" t="n">
+        <f aca="false">G26</f>
+        <v>6443597.89818208</v>
+      </c>
+      <c r="D41" s="36" t="n">
+        <f aca="false">C41-B41</f>
+        <v>1774668.42366797</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="13" t="s">
+        <v>253</v>
+      </c>
+      <c r="B42" s="35" t="n">
+        <f aca="false">SUM(B32:D32)/SUM(B33:D33)</f>
+        <v>1.15014090187089</v>
+      </c>
+      <c r="C42" s="35" t="n">
+        <f aca="false">SUM(E32:G32)/SUM(E33:G33)</f>
+        <v>1.74848671400674</v>
+      </c>
+      <c r="D42" s="38" t="n">
+        <f aca="false">C42-B42</f>
+        <v>0.598345812135851</v>
+      </c>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="2" t="s">
+        <v>254</v>
+      </c>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="3" t="s">
+        <v>255</v>
+      </c>
+      <c r="B45" s="3" t="s">
+        <v>256</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>257</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="13" t="s">
+        <v>81</v>
+      </c>
+      <c r="B46" s="13" t="s">
+        <v>258</v>
+      </c>
+      <c r="C46" s="13" t="s">
+        <v>258</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B47" s="20" t="n">
+        <f aca="false">$B$7^(1-1)*$B$11*($B$8*(1+$B$10)^1+$B$9*((1+$B$10)^1-1)/$B$10)+$B$12*$B$13*$B$14+$B$15*$B$16*$B$17</f>
+        <v>1208.574875</v>
+      </c>
+      <c r="C47" s="20" t="n">
+        <f aca="false">$C$7^(1-1)*$C$11*($C$8*(1+$C$10)^1+$C$9*((1+$C$10)^1-1)/$C$10)+$C$12*$C$13*$C$14+$C$15*$C$16*$C$17</f>
+        <v>1393.574875</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B48" s="20" t="n">
+        <f aca="false">$B$7^(2-1)*$B$11*($B$8*(1+$B$10)^2+$B$9*((1+$B$10)^2-1)/$B$10)+$B$7^(2-1)*$B$15*$B$16*$B$18</f>
+        <v>469.496730614438</v>
+      </c>
+      <c r="C48" s="20" t="n">
+        <f aca="false">$C$7^(2-1)*$C$11*($C$8*(1+$C$10)^2+$C$9*((1+$C$10)^2-1)/$C$10)+$C$7^(2-1)*$C$15*$C$16*$C$18</f>
+        <v>488.368906612735</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="B49" s="20" t="n">
+        <f aca="false">$B$7^(3-1)*$B$11*($B$8*(1+$B$10)^3+$B$9*((1+$B$10)^3-1)/$B$10)+$B$7^(3-1)*$B$15*$B$16*$B$18</f>
+        <v>506.140362986786</v>
+      </c>
+      <c r="C49" s="20" t="n">
+        <f aca="false">$C$7^(3-1)*$C$11*($C$8*(1+$C$10)^3+$C$9*((1+$C$10)^3-1)/$C$10)+$C$7^(3-1)*$C$15*$C$16*$C$18</f>
+        <v>543.072084824639</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="B50" s="20" t="n">
+        <f aca="false">$B$7^(4-1)*$B$11*($B$8*(1+$B$10)^4+$B$9*((1+$B$10)^4-1)/$B$10)+$B$7^(4-1)*$B$15*$B$16*$B$18</f>
+        <v>537.758819559933</v>
+      </c>
+      <c r="C50" s="20" t="n">
+        <f aca="false">$C$7^(4-1)*$C$11*($C$8*(1+$C$10)^4+$C$9*((1+$C$10)^4-1)/$C$10)+$C$7^(4-1)*$C$15*$C$16*$C$18</f>
+        <v>595.314903414714</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="B51" s="20" t="n">
+        <f aca="false">$B$7^(5-1)*$B$11*($B$8*(1+$B$10)^5+$B$9*((1+$B$10)^5-1)/$B$10)+$B$7^(5-1)*$B$15*$B$16*$B$18</f>
+        <v>564.813188772839</v>
+      </c>
+      <c r="C51" s="20" t="n">
+        <f aca="false">$C$7^(5-1)*$C$11*($C$8*(1+$C$10)^5+$C$9*((1+$C$10)^5-1)/$C$10)+$C$7^(5-1)*$C$15*$C$16*$C$18</f>
+        <v>645.221334776332</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="B52" s="20" t="n">
+        <f aca="false">$B$7^(6-1)*$B$11*($B$8*(1+$B$10)^6+$B$9*((1+$B$10)^6-1)/$B$10)+$B$7^(6-1)*$B$15*$B$16*$B$18</f>
+        <v>587.726005176324</v>
+      </c>
+      <c r="C52" s="20" t="n">
+        <f aca="false">$C$7^(6-1)*$C$11*($C$8*(1+$C$10)^6+$C$9*((1+$C$10)^6-1)/$C$10)+$C$7^(6-1)*$C$15*$C$16*$C$18</f>
+        <v>692.909155997988</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="4" t="n">
+        <v>7</v>
+      </c>
+      <c r="B53" s="20" t="n">
+        <f aca="false">$B$7^(7-1)*$B$11*($B$8*(1+$B$10)^7+$B$9*((1+$B$10)^7-1)/$B$10)+$B$7^(7-1)*$B$15*$B$16*$B$18</f>
+        <v>606.88438077407</v>
+      </c>
+      <c r="C53" s="20" t="n">
+        <f aca="false">$C$7^(7-1)*$C$11*($C$8*(1+$C$10)^7+$C$9*((1+$C$10)^7-1)/$C$10)+$C$7^(7-1)*$C$15*$C$16*$C$18</f>
+        <v>738.490258640058</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="B54" s="20" t="n">
+        <f aca="false">$B$7^(8-1)*$B$11*($B$8*(1+$B$10)^8+$B$9*((1+$B$10)^8-1)/$B$10)+$B$7^(8-1)*$B$15*$B$16*$B$18</f>
+        <v>622.642884529396</v>
+      </c>
+      <c r="C54" s="20" t="n">
+        <f aca="false">$C$7^(8-1)*$C$11*($C$8*(1+$C$10)^8+$C$9*((1+$C$10)^8-1)/$C$10)+$C$7^(8-1)*$C$15*$C$16*$C$18</f>
+        <v>782.07094302276</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="B55" s="20" t="n">
+        <f aca="false">$B$7^(9-1)*$B$11*($B$8*(1+$B$10)^9+$B$9*((1+$B$10)^9-1)/$B$10)+$B$7^(9-1)*$B$15*$B$16*$B$18</f>
+        <v>635.326190221928</v>
+      </c>
+      <c r="C55" s="20" t="n">
+        <f aca="false">$C$7^(9-1)*$C$11*($C$8*(1+$C$10)^9+$C$9*((1+$C$10)^9-1)/$C$10)+$C$7^(9-1)*$C$15*$C$16*$C$18</f>
+        <v>823.75219779975</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="4" t="n">
+        <v>10</v>
+      </c>
+      <c r="B56" s="20" t="n">
+        <f aca="false">$B$7^(10-1)*$B$11*($B$8*(1+$B$10)^10+$B$9*((1+$B$10)^10-1)/$B$10)+$B$7^(10-1)*$B$15*$B$16*$B$18</f>
+        <v>645.231511222615</v>
+      </c>
+      <c r="C56" s="20" t="n">
+        <f aca="false">$C$7^(10-1)*$C$11*($C$8*(1+$C$10)^10+$C$9*((1+$C$10)^10-1)/$C$10)+$C$7^(10-1)*$C$15*$C$16*$C$18</f>
+        <v>863.629965553088</v>
+      </c>
+      <c r="D56" s="13" t="s">
+        <v>248</v>
+      </c>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="13" t="s">
+        <v>259</v>
+      </c>
+      <c r="B57" s="36" t="n">
+        <f aca="false">NPV($B$20,B47:B56)</f>
+        <v>4380.59143972022</v>
+      </c>
+      <c r="C57" s="36" t="n">
+        <f aca="false">NPV($C$20,C47:C56)</f>
+        <v>5119.04371900083</v>
+      </c>
+      <c r="D57" s="36" t="n">
+        <f aca="false">C57-B57</f>
+        <v>738.452279280609</v>
+      </c>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="13" t="s">
+        <v>260</v>
+      </c>
+      <c r="B58" s="36" t="n">
+        <f aca="false">B57*B23</f>
+        <v>157701.291829928</v>
+      </c>
+      <c r="C58" s="36" t="n">
+        <f aca="false">C57*E23</f>
+        <v>245714.09851204</v>
+      </c>
+      <c r="D58" s="36" t="n">
+        <f aca="false">C58-B58</f>
+        <v>88012.8066821119</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="2" t="s">
+        <v>261</v>
       </c>
     </row>
   </sheetData>

</xml_diff>